<commit_message>
Add fraud ranking file
</commit_message>
<xml_diff>
--- a/analysis/Fraud Ranking For Channel and Txn Types.xlsx
+++ b/analysis/Fraud Ranking For Channel and Txn Types.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Jazzcash\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Jazzcash\jazzcash-fraud-detection\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -54087,7 +54087,7 @@
         <v>8</v>
       </c>
       <c r="D130" s="37">
-        <f t="shared" ref="D130:D161" si="9">C130/$C$153</f>
+        <f t="shared" ref="D130:D152" si="9">C130/$C$153</f>
         <v>6.3842864833642248E-7</v>
       </c>
       <c r="E130" s="81">

</xml_diff>